<commit_message>
Upgrade LCD to OLED
</commit_message>
<xml_diff>
--- a/wizardry/pin_defs.xlsx
+++ b/wizardry/pin_defs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\Documents\Projects\Ongoing\Progtomata\wizardry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\henri\Projects\Ongoing\EmbeddedSystems\Software\Progtomata\wizardry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8CB5B4-DAFA-455F-8AFB-93554D8608A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC4CDCB-7C08-498A-8CC9-8196F0B7D8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="102">
   <si>
     <t>P1</t>
   </si>
@@ -293,18 +293,6 @@
   </si>
   <si>
     <t>LCD_EN</t>
-  </si>
-  <si>
-    <t>LCD_D4</t>
-  </si>
-  <si>
-    <t>LCD_D5</t>
-  </si>
-  <si>
-    <t>LCD_D6</t>
-  </si>
-  <si>
-    <t>LCD_D7</t>
   </si>
   <si>
     <t>ENC1_Q0</t>
@@ -509,6 +497,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -526,9 +517,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -845,18 +833,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="7"/>
-      <c r="F1" s="8" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="8"/>
+      <c r="F1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -971,13 +959,13 @@
         <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>54</v>
@@ -1041,13 +1029,13 @@
         <v>58</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>82</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1114,9 +1102,7 @@
       <c r="C15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="D15" s="1"/>
       <c r="F15" s="4" t="s">
         <v>62</v>
       </c>
@@ -1130,15 +1116,11 @@
       <c r="A16" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>92</v>
-      </c>
+      <c r="B16" s="1"/>
       <c r="C16" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>93</v>
-      </c>
+      <c r="D16" s="1"/>
       <c r="F16" s="4" t="s">
         <v>66</v>
       </c>
@@ -1152,9 +1134,7 @@
       <c r="A17" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>94</v>
-      </c>
+      <c r="B17" s="1"/>
       <c r="C17" s="4" t="s">
         <v>42</v>
       </c>
@@ -1181,13 +1161,13 @@
         <v>74</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>81</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -1217,7 +1197,7 @@
         <v>24</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>76</v>
@@ -1233,7 +1213,7 @@
         <v>25</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>26</v>
@@ -1247,7 +1227,7 @@
         <v>67</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -1281,13 +1261,13 @@
         <v>70</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>69</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
@@ -1345,10 +1325,10 @@
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N27" s="11"/>
+      <c r="N27" s="5"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N28" s="11"/>
+      <c r="N28" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>